<commit_message>
CS575 Homework 2 File Changes
</commit_message>
<xml_diff>
--- a/BU/CS575/Homework 2/System Calls.xlsx
+++ b/BU/CS575/Homework 2/System Calls.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jirissman/Documents/coursework/BU/CS575/Homework 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C681B3D-A868-7748-A68E-D521AFCB741D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E384F13B-4B00-224D-854C-FCBECE9FE4BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{B3284229-6A5E-AE4C-9202-662B9D044611}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" xr2:uid="{B3284229-6A5E-AE4C-9202-662B9D044611}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>System Calls</t>
   </si>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>"strace -e" output file size</t>
-  </si>
-  <si>
-    <t>To find size use "ls -ltrh"</t>
   </si>
   <si>
     <t>1.1K</t>
@@ -116,7 +113,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -124,12 +121,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,171 +495,175 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="4">
         <v>5</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="4">
         <v>21</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="4">
         <v>42</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="4">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="4">
         <v>2</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="4">
         <v>5</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="4">
         <v>10</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="4">
         <v>37</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="4">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="4">
         <v>9</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="4">
         <v>50</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="4">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
+      <c r="B6" s="4">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4">
         <v>0</v>
       </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="4">
         <v>6</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="4">
         <v>18</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="4">
         <v>29</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="4">
         <v>23</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F8" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CS757 Homework 2 File Changes
</commit_message>
<xml_diff>
--- a/BU/CS575/Homework 2/System Calls.xlsx
+++ b/BU/CS575/Homework 2/System Calls.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jirissman/Documents/coursework/BU/CS575/Homework 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C681B3D-A868-7748-A68E-D521AFCB741D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E384F13B-4B00-224D-854C-FCBECE9FE4BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{B3284229-6A5E-AE4C-9202-662B9D044611}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16660" xr2:uid="{B3284229-6A5E-AE4C-9202-662B9D044611}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>System Calls</t>
   </si>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>"strace -e" output file size</t>
-  </si>
-  <si>
-    <t>To find size use "ls -ltrh"</t>
   </si>
   <si>
     <t>1.1K</t>
@@ -116,7 +113,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -124,12 +121,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,171 +495,175 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="4">
         <v>5</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="4">
         <v>21</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="4">
         <v>42</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="4">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="4">
         <v>2</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="4">
         <v>5</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="4">
         <v>10</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="4">
         <v>37</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="4">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="4">
         <v>9</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="4">
         <v>50</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="4">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
+      <c r="B6" s="4">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4">
         <v>0</v>
       </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="4">
         <v>6</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="4">
         <v>18</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="4">
         <v>29</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="4">
         <v>23</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F8" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>